<commit_message>
chore: overwrite 露天.xlsx via Streamlit restore
</commit_message>
<xml_diff>
--- a/data/露天.xlsx
+++ b/data/露天.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z1"/>
+  <dimension ref="A1:Z8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -545,6 +545,744 @@
       <c r="Z1" t="inlineStr">
         <is>
           <t>收件地址</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026/01/20</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>26012044321148</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>萊爾富取貨付款</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>jimshue</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>22212317280954</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>『單顆入』好評銷售冠軍👑台灣天然養生手工黑糖塊｜老薑紅棗桂圓海燕窩｜冬日暖身｜生理期保養｜暖男送女友必備🎁｜黑糖磚</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>老薑黑糖塊</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>YGJ03002-OG</t>
+        </is>
+      </c>
+      <c r="L2" t="n">
+        <v>10</v>
+      </c>
+      <c r="M2" t="n">
+        <v>10</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>萊爾富取貨付款</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>17</v>
+      </c>
+      <c r="S2" t="n">
+        <v>83</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/26&lt;br&gt;01/24 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>26DME37477238</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>許*誠</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026/01/13</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>26011343534591</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>x200129</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>寶藍色</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>L ➜建議70-75KG</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>HME03001-PB-L</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>3</v>
+      </c>
+      <c r="M3" t="n">
+        <v>67</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1005</v>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/15&lt;br&gt;01/15 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>M51801615754</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>朱*慶</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026/01/13</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>26011343534591</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>x200129</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>咖啡色</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>L ➜建議70-75KG</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>HME03001-BR-L</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>3</v>
+      </c>
+      <c r="M4" t="n">
+        <v>67</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1005</v>
+      </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/15&lt;br&gt;01/15 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>M51801615754</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>朱*慶</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026/01/13</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>26011343534591</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>x200129</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>灰色</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>L ➜建議70-75KG</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>HME03001-GY-L</t>
+        </is>
+      </c>
+      <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
+        <v>67</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S5" t="n">
+        <v>1005</v>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/15&lt;br&gt;01/15 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V5" t="inlineStr">
+        <is>
+          <t>M51801615754</t>
+        </is>
+      </c>
+      <c r="W5" t="inlineStr">
+        <is>
+          <t>朱*慶</t>
+        </is>
+      </c>
+      <c r="X5" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z5" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026/01/13</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26011343534591</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>x200129</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>酒紅色</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>L ➜建議70-75KG</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>HME03001-RD-L</t>
+        </is>
+      </c>
+      <c r="L6" t="n">
+        <v>3</v>
+      </c>
+      <c r="M6" t="n">
+        <v>67</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="O6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S6" t="n">
+        <v>1005</v>
+      </c>
+      <c r="T6" t="inlineStr"/>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/15&lt;br&gt;01/15 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V6" t="inlineStr">
+        <is>
+          <t>M51801615754</t>
+        </is>
+      </c>
+      <c r="W6" t="inlineStr">
+        <is>
+          <t>朱*慶</t>
+        </is>
+      </c>
+      <c r="X6" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y6" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z6" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026/01/13</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>26011343534591</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>x200129</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>黑色</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>L ➜建議70-75KG</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>HME03001-BK-L</t>
+        </is>
+      </c>
+      <c r="L7" t="n">
+        <v>3</v>
+      </c>
+      <c r="M7" t="n">
+        <v>67</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>7-11取貨付款</t>
+        </is>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>1005</v>
+      </c>
+      <c r="T7" t="inlineStr"/>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/15&lt;br&gt;01/15 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>M51801615754</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>朱*慶</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026/01/10</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>26011043215466</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>已出貨</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>全家取貨付款</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>superart</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>21828333346889</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>[台灣冠軍🏆爆賣30萬件]冰絲內褲 男內褲 涼感內褲 男士內褲 平口褲</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>黑色</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>S ➜建議50-55KG</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>HME03001-BK-S</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M8" t="n">
+        <v>67</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>全家取貨付款</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>30</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>365</v>
+      </c>
+      <c r="T8" t="inlineStr"/>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>訂單完成&lt;br&gt;2026/01/27&lt;br&gt;01/12 買家已取貨</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>16327964981</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>邱*慶</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>**********</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>**********</t>
         </is>
       </c>
     </row>

</xml_diff>